<commit_message>
Otomatik veri güncelleme (30.10.2026 17:15 UTC)
</commit_message>
<xml_diff>
--- a/net rezerv/likidite.xlsx
+++ b/net rezerv/likidite.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1377,6 +1377,29 @@
         <v>-12170</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="1" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B42" t="n">
+        <v>162191</v>
+      </c>
+      <c r="C42" t="n">
+        <v>51376</v>
+      </c>
+      <c r="D42" t="n">
+        <v>103146</v>
+      </c>
+      <c r="E42" t="n">
+        <v>-16489</v>
+      </c>
+      <c r="F42" t="n">
+        <v>4382</v>
+      </c>
+      <c r="G42" t="n">
+        <v>-12107</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>